<commit_message>
Negociações: tabela por mês e conferência com o valor do Power BI
- embaixo da tabela por equipe, a "Negociação por mês": total, valor e ticket médio de
  cada mês com negociação (do mais recente para o mais antigo) e o total; vale o filtro
  de equipe, não o de período
- "Diferenças com o Power BI" (só na tela): as negociações do período em que o valor do
  painel difere da fórmula do relatório (dígitos ÷ 100; texto com letras = R$ 0,00), com
  o texto original, os dois valores e o motivo. A contagem é a mesma; só o valor muda
- regras.negociacoes.igualPowerBI (padrão false) faz as contas com a fórmula do relatório
- Excel: aba "Negociação por mês" e coluna "Valor no Power BI (R$)"

165 testes (4 novos).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NfeRmDCrARwQbeV838mFqP
</commit_message>
<xml_diff>
--- a/exemplos/exemplo-negociacoes.xlsx
+++ b/exemplos/exemplo-negociacoes.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1081,6 +1081,118 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RIORECIN-007</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>80000012</v>
+      </c>
+      <c r="C13" t="n">
+        <v>100000212</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Verificação Cadastral</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>MIRACEMA</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>CENTRO</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>PROJETO VIDA NOVA: FAVOR IDENTIFICAR O CLIENTE E NEGOCIAR OS DEBITOS VENCIDOS.</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>À vista</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>R$ 238,23 em 3x</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RIOVENIN-002</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>80000013</v>
+      </c>
+      <c r="C14" t="n">
+        <v>100000213</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Verificação Cadastral</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>MIRACEMA</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>CENTRO</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>PROJETO VIDA NOVA: FAVOR IDENTIFICAR O CLIENTE E NEGOCIAR OS DEBITOS VENCIDOS.</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>À vista</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>R$ 300</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Negociações: sem "Valor Total dos Débitos", o valor vem do Parecer De Campo
Quando a negociação não tem "Valor Total dos Débitos" (vazio ou sem número), o painel
procura o valor no "Parecer De Campo": o primeiro com "R$" na frente ou, sem "R$", o
primeiro no formato 1.234,56 (normalize.valorNoTexto).

- a tela avisa quantas tiveram o valor tirado do parecer e quantas seguem sem valor
- Excel: Parecer De Campo, valor no parecer e origem do valor em cada negociação;
  "Valor tirado do Parecer" nas abas por equipe e por mês
- as Atividades passam a guardar o valor do parecer das negociações (antes o parecer
  ficava cortado): os dados do navegador são relidos da pasta uma vez (só no Interior)

166 testes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NfeRmDCrARwQbeV838mFqP
</commit_message>
<xml_diff>
--- a/exemplos/exemplo-negociacoes.xlsx
+++ b/exemplos/exemplo-negociacoes.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,6 +481,11 @@
           <t>Valor Total dos Débitos</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Parecer De Campo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -537,6 +542,11 @@
           <t>R$ 1.234,56</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -593,6 +603,11 @@
           <t>645,15</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -649,6 +664,11 @@
           <t>R$ 120,29</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -703,6 +723,11 @@
       <c r="L5" t="n">
         <v>1000.5</v>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -754,6 +779,11 @@
           <t>À vista</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Cliente negociou o débito de R$ 812,40 em 6x de R$ 135,40, leitura 1234,56.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -810,6 +840,11 @@
           <t>R$ 900,00</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -866,6 +901,11 @@
           <t>R$ 300,00</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -922,6 +962,11 @@
           <t>R$ 5.000,00</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -978,6 +1023,11 @@
           <t>1234.5</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1034,6 +1084,11 @@
           <t>R$ 200,00</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1080,6 +1135,11 @@
           <t>R$ 50,00</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1136,6 +1196,11 @@
           <t>R$ 238,23 em 3x</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1190,6 +1255,123 @@
       <c r="L14" t="inlineStr">
         <is>
           <t>R$ 300</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Cliente atendido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RIORECIN-004</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>80000014</v>
+      </c>
+      <c r="C15" t="n">
+        <v>100000214</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Verificação Cadastral</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>MIRACEMA</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>CENTRO</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>PROJETO VIDA NOVA: FAVOR IDENTIFICAR O CLIENTE E NEGOCIAR OS DEBITOS VENCIDOS.</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>À vista</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Negociado, cliente vai pagar na agência dia 10/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>RIORECIN-007</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>80000015</v>
+      </c>
+      <c r="C16" t="n">
+        <v>100000215</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Verificação Cadastral</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>MIRACEMA</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>CENTRO</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>PROJETO VIDA NOVA: FAVOR IDENTIFICAR O CLIENTE E NEGOCIAR OS DEBITOS VENCIDOS.</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>À vista</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>DEBITO NEGOCIADO 1.250,00 ENTRADA 125,00</t>
         </is>
       </c>
     </row>

</xml_diff>